<commit_message>
Update Feature & Optimizing Function
</commit_message>
<xml_diff>
--- a/static/laporan_peminjaman.xlsx
+++ b/static/laporan_peminjaman.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Murid</t>
+          <t>Siswa</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -481,49 +481,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Filosofi Teras</t>
+          <t>Atomic Habits</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Kembali</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Yusra</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Murid</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>XI</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>RPL</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Filosofi Teras</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Dipinjam</t>
+          <t>Selesai (Rusak)</t>
         </is>
       </c>
     </row>

</xml_diff>